<commit_message>
Correction num_instrument dans Recolteur&instrument_projet
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_projets.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_projets.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Projet" sheetId="1" state="visible" r:id="rId3"/>
@@ -183,10 +183,10 @@
     <t xml:space="preserve">HOBO_n°38</t>
   </si>
   <si>
-    <t xml:space="preserve">TMS4_n°0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dendro_n°0</t>
+    <t xml:space="preserve">TMS4_95224601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dendro_92261195</t>
   </si>
   <si>
     <t xml:space="preserve">id_groupe_recolte</t>
@@ -203,7 +203,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -239,6 +239,12 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -283,7 +289,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -305,6 +311,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1033,7 +1043,7 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="6" t="s">
         <v>53</v>
       </c>
       <c r="B42" s="1" t="n">
@@ -1044,10 +1054,10 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="1" t="s">
+      <c r="A43" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B43" s="0" t="n">
+      <c r="B43" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">

</xml_diff>